<commit_message>
init: images and latex init
</commit_message>
<xml_diff>
--- a/project/stage03/analysis.xlsx
+++ b/project/stage03/analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jantar\uni-data-warehouse\project\stage03\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C56ADF1-F630-4BEA-AB40-F38E3150B910}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66B34051-7248-439E-BC57-6979ECC90A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="879" firstSheet="5" activeTab="9" xr2:uid="{5D7D4CC1-6A94-48C8-A9CB-AB14AE6EE489}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="879" firstSheet="1" activeTab="5" xr2:uid="{5D7D4CC1-6A94-48C8-A9CB-AB14AE6EE489}"/>
   </bookViews>
   <sheets>
     <sheet name="RainVsPitStops" sheetId="1" r:id="rId1"/>
@@ -26,20 +26,20 @@
   </sheets>
   <calcPr calcId="0"/>
   <pivotCaches>
-    <pivotCache cacheId="398" r:id="rId11"/>
-    <pivotCache cacheId="401" r:id="rId12"/>
-    <pivotCache cacheId="404" r:id="rId13"/>
-    <pivotCache cacheId="407" r:id="rId14"/>
-    <pivotCache cacheId="410" r:id="rId15"/>
-    <pivotCache cacheId="413" r:id="rId16"/>
-    <pivotCache cacheId="416" r:id="rId17"/>
-    <pivotCache cacheId="419" r:id="rId18"/>
-    <pivotCache cacheId="422" r:id="rId19"/>
-    <pivotCache cacheId="425" r:id="rId20"/>
-    <pivotCache cacheId="428" r:id="rId21"/>
-    <pivotCache cacheId="431" r:id="rId22"/>
-    <pivotCache cacheId="434" r:id="rId23"/>
-    <pivotCache cacheId="440" r:id="rId24"/>
+    <pivotCache cacheId="0" r:id="rId11"/>
+    <pivotCache cacheId="1" r:id="rId12"/>
+    <pivotCache cacheId="2" r:id="rId13"/>
+    <pivotCache cacheId="3" r:id="rId14"/>
+    <pivotCache cacheId="4" r:id="rId15"/>
+    <pivotCache cacheId="5" r:id="rId16"/>
+    <pivotCache cacheId="6" r:id="rId17"/>
+    <pivotCache cacheId="7" r:id="rId18"/>
+    <pivotCache cacheId="8" r:id="rId19"/>
+    <pivotCache cacheId="9" r:id="rId20"/>
+    <pivotCache cacheId="10" r:id="rId21"/>
+    <pivotCache cacheId="11" r:id="rId22"/>
+    <pivotCache cacheId="12" r:id="rId23"/>
+    <pivotCache cacheId="13" r:id="rId24"/>
   </pivotCaches>
 </workbook>
 </file>
@@ -1344,7 +1344,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1358,7 +1358,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
@@ -2514,7 +2513,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="pl-PL"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -2713,6 +2712,20 @@
           <a:effectLst/>
         </c:spPr>
       </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="10"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
     </c:pivotFmts>
     <c:plotArea>
       <c:layout/>
@@ -2746,6 +2759,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-A57B-4A24-9AEC-ECB739D7B8A7}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -4204,7 +4222,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="pl-PL"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -4213,6 +4231,9 @@
       <c:pivotFmt>
         <c:idx val="0"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -4269,6 +4290,9 @@
       <c:pivotFmt>
         <c:idx val="1"/>
         <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -17477,6 +17501,7 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="536128527"/>
+        <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -18291,6 +18316,7 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="532057039"/>
+        <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -18469,7 +18495,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="pl-PL"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -18522,7 +18548,6 @@
               <a:endParaRPr lang="pl-PL"/>
             </a:p>
           </c:txPr>
-          <c:dLblPos val="bestFit"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
           <c:showCatName val="0"/>
@@ -18533,6 +18558,146 @@
             <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
           </c:extLst>
         </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="3"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="4"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="5"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="6"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="7"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="8"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="9"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="10"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln w="19050">
+            <a:solidFill>
+              <a:schemeClr val="lt1"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
       </c:pivotFmt>
     </c:pivotFmts>
     <c:plotArea>
@@ -18567,6 +18732,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-CCF9-42E0-A89B-3C53AED1CB29}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -18582,6 +18752,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-CCF9-42E0-A89B-3C53AED1CB29}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
@@ -18597,6 +18772,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-CCF9-42E0-A89B-3C53AED1CB29}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="3"/>
@@ -18612,6 +18792,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000007-CCF9-42E0-A89B-3C53AED1CB29}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="4"/>
@@ -18627,6 +18812,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000009-CCF9-42E0-A89B-3C53AED1CB29}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="5"/>
@@ -18642,6 +18832,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000B-CCF9-42E0-A89B-3C53AED1CB29}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="6"/>
@@ -18659,6 +18854,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000D-CCF9-42E0-A89B-3C53AED1CB29}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="7"/>
@@ -18676,6 +18876,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000F-CCF9-42E0-A89B-3C53AED1CB29}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="8"/>
@@ -18693,6 +18898,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000011-CCF9-42E0-A89B-3C53AED1CB29}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="9"/>
@@ -18710,6 +18920,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000013-CCF9-42E0-A89B-3C53AED1CB29}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:cat>
             <c:strRef>
@@ -18795,7 +19010,6 @@
           </c:extLst>
         </c:ser>
         <c:dLbls>
-          <c:dLblPos val="bestFit"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
           <c:showCatName val="0"/>
@@ -25685,13 +25899,13 @@
       <xdr:col>3</xdr:col>
       <xdr:colOff>142875</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>128586</xdr:rowOff>
+      <xdr:rowOff>128585</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>733425</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>133349</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>437030</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>134470</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -28425,7 +28639,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{56F7BB47-9FE9-44F6-BAE3-68381FD572F9}" name="PivotTable1" cacheId="428" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{56F7BB47-9FE9-44F6-BAE3-68381FD572F9}" name="PivotTable1" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" fieldListSortAscending="1">
   <location ref="A4:D12" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="7">
     <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
@@ -28682,7 +28896,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable10.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{64550925-18BC-4527-BBCE-E54A3262D0D6}" name="PivotTable1" cacheId="407" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{64550925-18BC-4527-BBCE-E54A3262D0D6}" name="PivotTable1" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" fieldListSortAscending="1">
   <location ref="A1:C7" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -28854,225 +29068,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable11.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5AA7137E-FDF2-411F-A7E9-D7AEEDDD54ED}" name="PivotTable4" cacheId="401" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1" fieldListSortAscending="1">
-  <location ref="F5:G16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="3" colPageCount="1"/>
-  <pivotFields count="5">
-    <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" measureFilter="1" sortType="descending" defaultSubtotal="0" defaultAttributeDrillState="1">
-      <items count="10">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-      </items>
-      <autoSortScope>
-        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
-          <references count="1">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </autoSortScope>
-    </pivotField>
-    <pivotField axis="axisPage" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1"/>
-    <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField axis="axisPage" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1"/>
-    <pivotField axis="axisPage" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="11">
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <pageFields count="3">
-    <pageField fld="1" hier="25" name="[Dim Status].[Status Category].&amp;[Mechanical Failure]" cap="Mechanical Failure"/>
-    <pageField fld="3" hier="37" name="[Dim Time].[Year].&amp;[2010]" cap="2010"/>
-    <pageField fld="4" hier="12" name="[Dim Constructor].[Continent].&amp;[Europe]" cap="Europe"/>
-  </pageFields>
-  <dataFields count="1">
-    <dataField fld="2" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="1">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotHierarchies count="78">
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy multipleItemSelectionAllowed="1">
-      <members count="1" level="1">
-        <member name="[Dim Constructor].[Continent].&amp;[Europe]"/>
-      </members>
-    </pivotHierarchy>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy multipleItemSelectionAllowed="1">
-      <members count="1" level="1">
-        <member name="[Dim Status].[Status Category].&amp;[Mechanical Failure]"/>
-      </members>
-    </pivotHierarchy>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy multipleItemSelectionAllowed="1">
-      <members count="11" level="1">
-        <member name="[Dim Time].[Year].&amp;[2010]"/>
-        <member name="[Dim Time].[Year].&amp;[2011]"/>
-        <member name="[Dim Time].[Year].&amp;[2012]"/>
-        <member name="[Dim Time].[Year].&amp;[2013]"/>
-        <member name="[Dim Time].[Year].&amp;[2014]"/>
-        <member name="[Dim Time].[Year].&amp;[2015]"/>
-        <member name="[Dim Time].[Year].&amp;[2016]"/>
-        <member name="[Dim Time].[Year].&amp;[2017]"/>
-        <member name="[Dim Time].[Year].&amp;[2018]"/>
-        <member name="[Dim Time].[Year].&amp;[2019]"/>
-        <member name="[Dim Time].[Year].&amp;[2020]"/>
-      </members>
-    </pivotHierarchy>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-  </pivotHierarchies>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <filters count="1">
-    <filter fld="0" type="count" id="1" iMeasureHier="53">
-      <autoFilter ref="A1">
-        <filterColumn colId="0">
-          <top10 val="10" filterVal="10"/>
-        </filterColumn>
-      </autoFilter>
-    </filter>
-  </filters>
-  <rowHierarchiesUsage count="1">
-    <rowHierarchyUsage hierarchyUsage="26"/>
-  </rowHierarchiesUsage>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" calculatedMembersInFilters="1" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable12.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A746FFF8-6B66-4252-8CEA-043143963F3D}" name="PivotTable3" cacheId="404" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A746FFF8-6B66-4252-8CEA-043143963F3D}" name="PivotTable3" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1" fieldListSortAscending="1">
   <location ref="A5:B16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="3" colPageCount="1"/>
   <pivotFields count="6">
     <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" measureFilter="1" sortType="descending" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -29153,7 +29149,7 @@
   <dataFields count="1">
     <dataField fld="2" baseField="0" baseItem="0"/>
   </dataFields>
-  <chartFormats count="10">
+  <chartFormats count="11">
     <chartFormat chart="0" format="0" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
@@ -29271,6 +29267,18 @@
         </references>
       </pivotArea>
     </chartFormat>
+    <chartFormat chart="0" format="10">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
   </chartFormats>
   <pivotHierarchies count="78">
     <pivotHierarchy/>
@@ -29335,6 +29343,344 @@
         <member name="[Dim Time].[Year].&amp;[1958]"/>
         <member name="[Dim Time].[Year].&amp;[1959]"/>
         <member name="[Dim Time].[Year].&amp;[1960]"/>
+      </members>
+    </pivotHierarchy>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+  </pivotHierarchies>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <filters count="1">
+    <filter fld="0" type="count" id="1" iMeasureHier="53">
+      <autoFilter ref="A1">
+        <filterColumn colId="0">
+          <top10 val="10" filterVal="10"/>
+        </filterColumn>
+      </autoFilter>
+    </filter>
+  </filters>
+  <rowHierarchiesUsage count="1">
+    <rowHierarchyUsage hierarchyUsage="26"/>
+  </rowHierarchiesUsage>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" calculatedMembersInFilters="1" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable12.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5AA7137E-FDF2-411F-A7E9-D7AEEDDD54ED}" name="PivotTable4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1" fieldListSortAscending="1">
+  <location ref="F5:G16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="3" colPageCount="1"/>
+  <pivotFields count="5">
+    <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" measureFilter="1" sortType="descending" defaultSubtotal="0" defaultAttributeDrillState="1">
+      <items count="10">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField axis="axisPage" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1"/>
+    <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField axis="axisPage" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1"/>
+    <pivotField axis="axisPage" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="11">
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <pageFields count="3">
+    <pageField fld="1" hier="25" name="[Dim Status].[Status Category].&amp;[Mechanical Failure]" cap="Mechanical Failure"/>
+    <pageField fld="3" hier="37" name="[Dim Time].[Year].&amp;[2010]" cap="2010"/>
+    <pageField fld="4" hier="12" name="[Dim Constructor].[Continent].&amp;[Europe]" cap="Europe"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField fld="2" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="11">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="2">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="3">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="4">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="8"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="5">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="6"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="6">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="7">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="9"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="8">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="9">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="7"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="10">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="5"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotHierarchies count="78">
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy multipleItemSelectionAllowed="1">
+      <members count="1" level="1">
+        <member name="[Dim Constructor].[Continent].&amp;[Europe]"/>
+      </members>
+    </pivotHierarchy>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy multipleItemSelectionAllowed="1">
+      <members count="1" level="1">
+        <member name="[Dim Status].[Status Category].&amp;[Mechanical Failure]"/>
+      </members>
+    </pivotHierarchy>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy multipleItemSelectionAllowed="1">
+      <members count="11" level="1">
+        <member name="[Dim Time].[Year].&amp;[2010]"/>
+        <member name="[Dim Time].[Year].&amp;[2011]"/>
+        <member name="[Dim Time].[Year].&amp;[2012]"/>
+        <member name="[Dim Time].[Year].&amp;[2013]"/>
+        <member name="[Dim Time].[Year].&amp;[2014]"/>
+        <member name="[Dim Time].[Year].&amp;[2015]"/>
+        <member name="[Dim Time].[Year].&amp;[2016]"/>
+        <member name="[Dim Time].[Year].&amp;[2017]"/>
+        <member name="[Dim Time].[Year].&amp;[2018]"/>
+        <member name="[Dim Time].[Year].&amp;[2019]"/>
+        <member name="[Dim Time].[Year].&amp;[2020]"/>
       </members>
     </pivotHierarchy>
     <pivotHierarchy/>
@@ -29403,7 +29749,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable13.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8EE1C926-7098-4912-8FCE-3C5B6C4A9ADA}" name="PivotTable5" cacheId="398" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8EE1C926-7098-4912-8FCE-3C5B6C4A9ADA}" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" fieldListSortAscending="1">
   <location ref="A1:G7" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisCol" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -29653,7 +29999,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable14.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8B5532C8-184E-45A3-9671-D5D71185BFA5}" name="PivotTable6" cacheId="440" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8B5532C8-184E-45A3-9671-D5D71185BFA5}" name="PivotTable6" cacheId="13" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1" fieldListSortAscending="1">
   <location ref="A3:B78" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="3">
     <pivotField axis="axisPage" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1"/>
@@ -30087,7 +30433,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C46A81BC-8C75-4F76-8210-EEF5A83AF696}" name="PivotTable4" cacheId="431" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C46A81BC-8C75-4F76-8210-EEF5A83AF696}" name="PivotTable4" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10" fieldListSortAscending="1">
   <location ref="A4:B22" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="7">
     <pivotField axis="axisPage" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1"/>
@@ -30641,7 +30987,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{48529DB8-E948-488C-A714-CF42C15C483B}" name="PivotTable2" cacheId="419" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{48529DB8-E948-488C-A714-CF42C15C483B}" name="PivotTable2" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" fieldListSortAscending="1">
   <location ref="F34:G58" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="3">
     <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
@@ -30894,7 +31240,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0D28268D-F139-414C-88E2-408A6595ABF9}" name="PivotTable5" cacheId="416" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="15" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0D28268D-F139-414C-88E2-408A6595ABF9}" name="PivotTable5" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="15" fieldListSortAscending="1">
   <location ref="A3:G5" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="3">
     <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
@@ -31148,7 +31494,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F77C5366-9A19-47B5-8C19-F54DD5D444B7}" name="PivotTable4" cacheId="425" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F77C5366-9A19-47B5-8C19-F54DD5D444B7}" name="PivotTable4" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11" fieldListSortAscending="1">
   <location ref="K5:U14" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
   <pivotFields count="5">
     <pivotField axis="axisPage" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -31500,7 +31846,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2F74144B-8497-4A58-998A-35E2F835E367}" name="PivotTable1" cacheId="422" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2F74144B-8497-4A58-998A-35E2F835E367}" name="PivotTable1" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" fieldListSortAscending="1">
   <location ref="A4:B31" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
   <pivotFields count="4">
     <pivotField axis="axisPage" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -31761,7 +32107,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FA00D414-BC42-451C-9F10-3DB99A7CAD38}" name="PivotTable3" cacheId="413" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FA00D414-BC42-451C-9F10-3DB99A7CAD38}" name="PivotTable3" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1" fieldListSortAscending="1">
   <location ref="A5:B32" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
   <pivotFields count="4">
     <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -32069,7 +32415,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F4BABA1E-A83D-4CB8-B63A-6BD641FCE2BF}" name="PivotTable1" cacheId="410" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F4BABA1E-A83D-4CB8-B63A-6BD641FCE2BF}" name="PivotTable1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" fieldListSortAscending="1">
   <location ref="A1:C29" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -32323,7 +32669,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7F60A7DA-9FE7-47E8-A86B-C8A0C2243D7A}" name="PivotTable2" cacheId="434" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7F60A7DA-9FE7-47E8-A86B-C8A0C2243D7A}" name="PivotTable2" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" fieldListSortAscending="1">
   <location ref="A12:C18" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -32872,13 +33218,13 @@
       <c r="A6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6">
         <v>1.4611872146118721</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6">
         <v>1.3251533742331287</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6">
         <v>1.4031413612565444</v>
       </c>
     </row>
@@ -32886,13 +33232,13 @@
       <c r="A7" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7">
         <v>1.4928774928774928</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7">
         <v>2.1724137931034484</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7">
         <v>1.5892420537897312</v>
       </c>
     </row>
@@ -32900,13 +33246,13 @@
       <c r="A8" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8">
         <v>1.904040404040404</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C8">
         <v>1.9661016949152543</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8">
         <v>1.9182879377431907</v>
       </c>
     </row>
@@ -32914,13 +33260,13 @@
       <c r="A9" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B9">
         <v>1.9824561403508771</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C9">
         <v>2.36</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9">
         <v>2.0611111111111109</v>
       </c>
     </row>
@@ -32928,13 +33274,13 @@
       <c r="A10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="7">
+      <c r="B10">
         <v>1.9039735099337749</v>
       </c>
-      <c r="C10" s="7">
+      <c r="C10">
         <v>2.1296296296296298</v>
       </c>
-      <c r="D10" s="7">
+      <c r="D10">
         <v>1.9634146341463414</v>
       </c>
     </row>
@@ -32942,13 +33288,13 @@
       <c r="A11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="7">
+      <c r="B11">
         <v>1.8850931677018634</v>
       </c>
-      <c r="C11" s="7">
+      <c r="C11">
         <v>3.2105263157894739</v>
       </c>
-      <c r="D11" s="7">
+      <c r="D11">
         <v>2.1870503597122304</v>
       </c>
     </row>
@@ -32956,13 +33302,13 @@
       <c r="A12" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="7">
+      <c r="B12">
         <v>1.7698270721526534</v>
       </c>
-      <c r="C12" s="7">
+      <c r="C12">
         <v>2.096774193548387</v>
       </c>
-      <c r="D12" s="7">
+      <c r="D12">
         <v>1.8514541387024608</v>
       </c>
     </row>
@@ -33002,7 +33348,7 @@
       <c r="A4" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="7">
         <v>10335466.666666666</v>
       </c>
     </row>
@@ -33010,7 +33356,7 @@
       <c r="A5" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="7">
         <v>9771600</v>
       </c>
     </row>
@@ -33018,7 +33364,7 @@
       <c r="A6" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="7">
         <v>10324950</v>
       </c>
     </row>
@@ -33026,7 +33372,7 @@
       <c r="A7" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="7">
         <v>10186600</v>
       </c>
     </row>
@@ -33034,7 +33380,7 @@
       <c r="A8" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="B8" s="8">
+      <c r="B8" s="7">
         <v>10067900</v>
       </c>
     </row>
@@ -33042,7 +33388,7 @@
       <c r="A9" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="7">
         <v>8775500</v>
       </c>
     </row>
@@ -33050,7 +33396,7 @@
       <c r="A10" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10" s="7">
         <v>8625100</v>
       </c>
     </row>
@@ -33058,7 +33404,7 @@
       <c r="A11" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="B11" s="8">
+      <c r="B11" s="7">
         <v>9324500</v>
       </c>
     </row>
@@ -33066,7 +33412,7 @@
       <c r="A12" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="7">
         <v>7445300</v>
       </c>
     </row>
@@ -33074,7 +33420,7 @@
       <c r="A13" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="7">
         <v>7495100</v>
       </c>
     </row>
@@ -33082,7 +33428,7 @@
       <c r="A14" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="B14" s="8">
+      <c r="B14" s="7">
         <v>8543000</v>
       </c>
     </row>
@@ -33090,7 +33436,7 @@
       <c r="A15" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="B15" s="8">
+      <c r="B15" s="7">
         <v>7493100</v>
       </c>
     </row>
@@ -33098,7 +33444,7 @@
       <c r="A16" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="B16" s="8">
+      <c r="B16" s="7">
         <v>8995820</v>
       </c>
     </row>
@@ -33106,7 +33452,7 @@
       <c r="A17" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="B17" s="8">
+      <c r="B17" s="7">
         <v>8707100</v>
       </c>
     </row>
@@ -33114,7 +33460,7 @@
       <c r="A18" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="B18" s="8">
+      <c r="B18" s="7">
         <v>7884800</v>
       </c>
     </row>
@@ -33122,7 +33468,7 @@
       <c r="A19" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="B19" s="8">
+      <c r="B19" s="7">
         <v>7516725</v>
       </c>
     </row>
@@ -33130,7 +33476,7 @@
       <c r="A20" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="B20" s="8">
+      <c r="B20" s="7">
         <v>6438766.666666667</v>
       </c>
     </row>
@@ -33138,7 +33484,7 @@
       <c r="A21" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="B21" s="8">
+      <c r="B21" s="7">
         <v>6244975</v>
       </c>
     </row>
@@ -33146,7 +33492,7 @@
       <c r="A22" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="B22" s="8">
+      <c r="B22" s="7">
         <v>6073800</v>
       </c>
     </row>
@@ -33154,7 +33500,7 @@
       <c r="A23" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="B23" s="8">
+      <c r="B23" s="7">
         <v>5958036</v>
       </c>
     </row>
@@ -33162,7 +33508,7 @@
       <c r="A24" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="B24" s="8">
+      <c r="B24" s="7">
         <v>5961691.666666667</v>
       </c>
     </row>
@@ -33170,7 +33516,7 @@
       <c r="A25" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="B25" s="8">
+      <c r="B25" s="7">
         <v>4709468.5714285718</v>
       </c>
     </row>
@@ -33178,7 +33524,7 @@
       <c r="A26" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="B26" s="8">
+      <c r="B26" s="7">
         <v>5435316.666666667</v>
       </c>
     </row>
@@ -33186,7 +33532,7 @@
       <c r="A27" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="B27" s="8">
+      <c r="B27" s="7">
         <v>5393785.7142857146</v>
       </c>
     </row>
@@ -33194,7 +33540,7 @@
       <c r="A28" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="B28" s="8">
+      <c r="B28" s="7">
         <v>5004900</v>
       </c>
     </row>
@@ -33202,7 +33548,7 @@
       <c r="A29" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="B29" s="8">
+      <c r="B29" s="7">
         <v>5000583.333333333</v>
       </c>
     </row>
@@ -33210,7 +33556,7 @@
       <c r="A30" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="B30" s="8">
+      <c r="B30" s="7">
         <v>5472763.6363636367</v>
       </c>
     </row>
@@ -33218,7 +33564,7 @@
       <c r="A31" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="B31" s="8">
+      <c r="B31" s="7">
         <v>5300033.333333333</v>
       </c>
     </row>
@@ -33226,7 +33572,7 @@
       <c r="A32" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="B32" s="8">
+      <c r="B32" s="7">
         <v>4066579.0909090908</v>
       </c>
     </row>
@@ -33234,7 +33580,7 @@
       <c r="A33" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="B33" s="8">
+      <c r="B33" s="7">
         <v>4958081.4285714282</v>
       </c>
     </row>
@@ -33242,7 +33588,7 @@
       <c r="A34" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="B34" s="8">
+      <c r="B34" s="7">
         <v>5248934.2</v>
       </c>
     </row>
@@ -33250,7 +33596,7 @@
       <c r="A35" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="B35" s="8">
+      <c r="B35" s="7">
         <v>4983324.25</v>
       </c>
     </row>
@@ -33258,7 +33604,7 @@
       <c r="A36" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="B36" s="8">
+      <c r="B36" s="7">
         <v>5037734</v>
       </c>
     </row>
@@ -33266,7 +33612,7 @@
       <c r="A37" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="B37" s="8">
+      <c r="B37" s="7">
         <v>4841189.5</v>
       </c>
     </row>
@@ -33274,7 +33620,7 @@
       <c r="A38" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="B38" s="8">
+      <c r="B38" s="7">
         <v>4722609.5</v>
       </c>
     </row>
@@ -33282,7 +33628,7 @@
       <c r="A39" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="B39" s="8">
+      <c r="B39" s="7">
         <v>4684527</v>
       </c>
     </row>
@@ -33290,7 +33636,7 @@
       <c r="A40" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="B40" s="8">
+      <c r="B40" s="7">
         <v>4534194.833333333</v>
       </c>
     </row>
@@ -33298,7 +33644,7 @@
       <c r="A41" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="B41" s="8">
+      <c r="B41" s="7">
         <v>4703726.125</v>
       </c>
     </row>
@@ -33306,7 +33652,7 @@
       <c r="A42" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="B42" s="8">
+      <c r="B42" s="7">
         <v>4782805.75</v>
       </c>
     </row>
@@ -33314,7 +33660,7 @@
       <c r="A43" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="B43" s="8">
+      <c r="B43" s="7">
         <v>4708868.2</v>
       </c>
     </row>
@@ -33322,7 +33668,7 @@
       <c r="A44" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="B44" s="8">
+      <c r="B44" s="7">
         <v>4707697.5</v>
       </c>
     </row>
@@ -33330,7 +33676,7 @@
       <c r="A45" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="B45" s="8">
+      <c r="B45" s="7">
         <v>4739363.2</v>
       </c>
     </row>
@@ -33338,7 +33684,7 @@
       <c r="A46" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="B46" s="8">
+      <c r="B46" s="7">
         <v>4647515</v>
       </c>
     </row>
@@ -33346,7 +33692,7 @@
       <c r="A47" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="B47" s="8">
+      <c r="B47" s="7">
         <v>4716555.8</v>
       </c>
     </row>
@@ -33354,7 +33700,7 @@
       <c r="A48" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="B48" s="8">
+      <c r="B48" s="7">
         <v>4725496.75</v>
       </c>
     </row>
@@ -33362,7 +33708,7 @@
       <c r="A49" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="B49" s="8">
+      <c r="B49" s="7">
         <v>4714750.4000000004</v>
       </c>
     </row>
@@ -33370,7 +33716,7 @@
       <c r="A50" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="B50" s="8">
+      <c r="B50" s="7">
         <v>4646023.9090909092</v>
       </c>
     </row>
@@ -33378,7 +33724,7 @@
       <c r="A51" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="B51" s="8">
+      <c r="B51" s="7">
         <v>4674193.333333333</v>
       </c>
     </row>
@@ -33386,7 +33732,7 @@
       <c r="A52" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="B52" s="8">
+      <c r="B52" s="7">
         <v>4647590.9000000004</v>
       </c>
     </row>
@@ -33394,7 +33740,7 @@
       <c r="A53" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="B53" s="8">
+      <c r="B53" s="7">
         <v>5293787.833333333</v>
       </c>
     </row>
@@ -33402,7 +33748,7 @@
       <c r="A54" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="B54" s="8">
+      <c r="B54" s="7">
         <v>4659644.5714285718</v>
       </c>
     </row>
@@ -33410,7 +33756,7 @@
       <c r="A55" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="B55" s="8">
+      <c r="B55" s="7">
         <v>4635018.5999999996</v>
       </c>
     </row>
@@ -33418,7 +33764,7 @@
       <c r="A56" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="B56" s="8">
+      <c r="B56" s="7">
         <v>4471408.8</v>
       </c>
     </row>
@@ -33426,7 +33772,7 @@
       <c r="A57" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="B57" s="8">
+      <c r="B57" s="7">
         <v>4551856.7272727275</v>
       </c>
     </row>
@@ -33434,7 +33780,7 @@
       <c r="A58" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="B58" s="8">
+      <c r="B58" s="7">
         <v>4508729.0999999996</v>
       </c>
     </row>
@@ -33442,7 +33788,7 @@
       <c r="A59" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="B59" s="8">
+      <c r="B59" s="7">
         <v>4526991.7</v>
       </c>
     </row>
@@ -33450,7 +33796,7 @@
       <c r="A60" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="B60" s="8">
+      <c r="B60" s="7">
         <v>4767425</v>
       </c>
     </row>
@@ -33458,7 +33804,7 @@
       <c r="A61" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="B61" s="8">
+      <c r="B61" s="7">
         <v>5247373</v>
       </c>
     </row>
@@ -33466,7 +33812,7 @@
       <c r="A62" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="B62" s="8">
+      <c r="B62" s="7">
         <v>4651278.6363636367</v>
       </c>
     </row>
@@ -33474,7 +33820,7 @@
       <c r="A63" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="B63" s="8">
+      <c r="B63" s="7">
         <v>4621699.461538462</v>
       </c>
     </row>
@@ -33482,7 +33828,7 @@
       <c r="A64" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="B64" s="8">
+      <c r="B64" s="7">
         <v>4866103</v>
       </c>
     </row>
@@ -33490,7 +33836,7 @@
       <c r="A65" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="B65" s="8">
+      <c r="B65" s="7">
         <v>4816472.153846154</v>
       </c>
     </row>
@@ -33498,7 +33844,7 @@
       <c r="A66" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="B66" s="8">
+      <c r="B66" s="7">
         <v>4740358.4666666668</v>
       </c>
     </row>
@@ -33506,7 +33852,7 @@
       <c r="A67" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="B67" s="8">
+      <c r="B67" s="7">
         <v>4800346.076923077</v>
       </c>
     </row>
@@ -33514,7 +33860,7 @@
       <c r="A68" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="B68" s="8">
+      <c r="B68" s="7">
         <v>4724407.333333333</v>
       </c>
     </row>
@@ -33522,7 +33868,7 @@
       <c r="A69" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="B69" s="8">
+      <c r="B69" s="7">
         <v>4690428.4000000004</v>
       </c>
     </row>
@@ -33530,7 +33876,7 @@
       <c r="A70" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="B70" s="8">
+      <c r="B70" s="7">
         <v>4580867.444444444</v>
       </c>
     </row>
@@ -33538,7 +33884,7 @@
       <c r="A71" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B71" s="8">
+      <c r="B71" s="7">
         <v>4648709.444444444</v>
       </c>
     </row>
@@ -33546,7 +33892,7 @@
       <c r="A72" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B72" s="8">
+      <c r="B72" s="7">
         <v>4570080.375</v>
       </c>
     </row>
@@ -33554,7 +33900,7 @@
       <c r="A73" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B73" s="8">
+      <c r="B73" s="7">
         <v>6447325.8125</v>
       </c>
     </row>
@@ -33562,7 +33908,7 @@
       <c r="A74" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B74" s="8">
+      <c r="B74" s="7">
         <v>4931917.4666666668</v>
       </c>
     </row>
@@ -33570,7 +33916,7 @@
       <c r="A75" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B75" s="8">
+      <c r="B75" s="7">
         <v>4833085.166666667</v>
       </c>
     </row>
@@ -33578,7 +33924,7 @@
       <c r="A76" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B76" s="8">
+      <c r="B76" s="7">
         <v>4469108.9375</v>
       </c>
     </row>
@@ -33586,7 +33932,7 @@
       <c r="A77" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B77" s="8">
+      <c r="B77" s="7">
         <v>4523655.153846154</v>
       </c>
     </row>
@@ -33594,7 +33940,7 @@
       <c r="A78" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B78" s="8">
+      <c r="B78" s="7">
         <v>5245271.0078431377</v>
       </c>
     </row>
@@ -33658,19 +34004,17 @@
       <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="7"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="7"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7">
         <v>1.2086570477247502</v>
       </c>
     </row>
@@ -33678,13 +34022,12 @@
       <c r="A8" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="7"/>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B9">
         <v>0.56140350877192979</v>
       </c>
     </row>
@@ -33692,7 +34035,7 @@
       <c r="A10" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="B10" s="7">
+      <c r="B10">
         <v>3.4645390070921986</v>
       </c>
     </row>
@@ -33700,7 +34043,7 @@
       <c r="A11" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="B11" s="7">
+      <c r="B11">
         <v>1.4308426073131955</v>
       </c>
     </row>
@@ -33708,13 +34051,12 @@
       <c r="A12" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="7"/>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="B13" s="7">
+      <c r="B13">
         <v>1.1666666666666667</v>
       </c>
     </row>
@@ -33722,7 +34064,7 @@
       <c r="A14" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="B14" s="7">
+      <c r="B14">
         <v>4.2163742690058479</v>
       </c>
     </row>
@@ -33730,7 +34072,7 @@
       <c r="A15" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="B15" s="7">
+      <c r="B15">
         <v>2.6777546777546779</v>
       </c>
     </row>
@@ -33738,7 +34080,7 @@
       <c r="A16" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="B16" s="7">
+      <c r="B16">
         <v>1.1880952380952381</v>
       </c>
     </row>
@@ -33746,7 +34088,7 @@
       <c r="A17" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="B17" s="7">
+      <c r="B17">
         <v>1.0948616600790513</v>
       </c>
     </row>
@@ -33754,7 +34096,7 @@
       <c r="A18" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="B18" s="7">
+      <c r="B18">
         <v>0.94680851063829785</v>
       </c>
     </row>
@@ -33762,13 +34104,12 @@
       <c r="A19" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="7"/>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="B20" s="7">
+      <c r="B20">
         <v>2.3026737967914439</v>
       </c>
     </row>
@@ -33776,7 +34117,7 @@
       <c r="A21" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="B21" s="7">
+      <c r="B21">
         <v>0.98565573770491799</v>
       </c>
     </row>
@@ -33784,7 +34125,7 @@
       <c r="A22" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B22" s="7">
+      <c r="B22">
         <v>1.6894683372841179</v>
       </c>
     </row>
@@ -33852,22 +34193,22 @@
       <c r="A5" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5">
         <v>4.5844155844155843</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5">
         <v>5.6934426229508199</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5">
         <v>9.9909836065573767</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5">
         <v>12.158196721311475</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5">
         <v>12.445081967213115</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5">
         <v>9.7461449498843482</v>
       </c>
     </row>
@@ -33911,7 +34252,7 @@
       <c r="F35" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G35" s="7">
+      <c r="G35">
         <v>12.445081967213115</v>
       </c>
       <c r="J35" s="2" t="s">
@@ -33925,7 +34266,7 @@
       <c r="F36" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="G36" s="7">
+      <c r="G36">
         <v>12.158196721311475</v>
       </c>
       <c r="J36" s="2" t="s">
@@ -33939,7 +34280,7 @@
       <c r="F37" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="G37" s="7">
+      <c r="G37">
         <v>9.9909836065573767</v>
       </c>
       <c r="J37" s="2" t="s">
@@ -33953,7 +34294,7 @@
       <c r="F38" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="G38" s="7">
+      <c r="G38">
         <v>5.6934426229508199</v>
       </c>
     </row>
@@ -33961,7 +34302,7 @@
       <c r="F39" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="G39" s="7">
+      <c r="G39">
         <v>4.5844155844155843</v>
       </c>
     </row>
@@ -33969,7 +34310,7 @@
       <c r="F40" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="G40" s="7">
+      <c r="G40">
         <v>3.7236842105263159</v>
       </c>
     </row>
@@ -33977,7 +34318,7 @@
       <c r="F41" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="G41" s="7">
+      <c r="G41">
         <v>3.0649717514124295</v>
       </c>
     </row>
@@ -33985,7 +34326,7 @@
       <c r="F42" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="G42" s="7">
+      <c r="G42">
         <v>2.7666666666666666</v>
       </c>
     </row>
@@ -33993,7 +34334,7 @@
       <c r="F43" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G43" s="7">
+      <c r="G43">
         <v>2.7333333333333334</v>
       </c>
     </row>
@@ -34001,7 +34342,7 @@
       <c r="F44" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="G44" s="7">
+      <c r="G44">
         <v>2.5181159420289854</v>
       </c>
     </row>
@@ -34009,7 +34350,7 @@
       <c r="F45" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="G45" s="7">
+      <c r="G45">
         <v>1.8433734939759037</v>
       </c>
     </row>
@@ -34017,7 +34358,7 @@
       <c r="F46" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="G46" s="7">
+      <c r="G46">
         <v>1.6995073891625616</v>
       </c>
     </row>
@@ -34025,7 +34366,7 @@
       <c r="F47" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="G47" s="7">
+      <c r="G47">
         <v>1.1212121212121211</v>
       </c>
     </row>
@@ -34033,7 +34374,7 @@
       <c r="F48" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="G48" s="7">
+      <c r="G48">
         <v>0.91044776119402981</v>
       </c>
     </row>
@@ -34041,7 +34382,7 @@
       <c r="F49" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="G49" s="7">
+      <c r="G49">
         <v>0.83333333333333337</v>
       </c>
     </row>
@@ -34049,7 +34390,7 @@
       <c r="F50" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="G50" s="7">
+      <c r="G50">
         <v>0.77105263157894732</v>
       </c>
     </row>
@@ -34057,7 +34398,7 @@
       <c r="F51" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G51" s="7">
+      <c r="G51">
         <v>0.70673076923076927</v>
       </c>
     </row>
@@ -34065,7 +34406,7 @@
       <c r="F52" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="G52" s="7">
+      <c r="G52">
         <v>1.834862385321101E-2</v>
       </c>
     </row>
@@ -34073,7 +34414,7 @@
       <c r="F53" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="G53" s="7">
+      <c r="G53">
         <v>1.282051282051282E-2</v>
       </c>
     </row>
@@ -34081,7 +34422,7 @@
       <c r="F54" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="G54" s="7">
+      <c r="G54">
         <v>0</v>
       </c>
     </row>
@@ -34089,7 +34430,7 @@
       <c r="F55" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="G55" s="7">
+      <c r="G55">
         <v>0</v>
       </c>
     </row>
@@ -34097,7 +34438,7 @@
       <c r="F56" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G56" s="7">
+      <c r="G56">
         <v>0</v>
       </c>
     </row>
@@ -34105,7 +34446,7 @@
       <c r="F57" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G57" s="7">
+      <c r="G57">
         <v>0</v>
       </c>
     </row>
@@ -34113,7 +34454,7 @@
       <c r="F58" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="G58" s="7">
+      <c r="G58">
         <v>4.8117619639527653</v>
       </c>
     </row>
@@ -34795,7 +35136,7 @@
       <c r="A6" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6">
         <v>7.333333333333333</v>
       </c>
     </row>
@@ -34803,7 +35144,7 @@
       <c r="A7" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7">
         <v>10.857142857142858</v>
       </c>
     </row>
@@ -34811,7 +35152,7 @@
       <c r="A8" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8">
         <v>12.461538461538462</v>
       </c>
     </row>
@@ -34819,7 +35160,7 @@
       <c r="A9" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B9">
         <v>9.2666666666666675</v>
       </c>
     </row>
@@ -34827,7 +35168,7 @@
       <c r="A10" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B10" s="7">
+      <c r="B10">
         <v>6.7058823529411766</v>
       </c>
     </row>
@@ -34835,7 +35176,7 @@
       <c r="A11" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B11" s="7">
+      <c r="B11">
         <v>10</v>
       </c>
     </row>
@@ -34843,7 +35184,7 @@
       <c r="A12" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B12" s="7">
+      <c r="B12">
         <v>22.181818181818183</v>
       </c>
     </row>
@@ -34851,7 +35192,7 @@
       <c r="A13" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="7">
+      <c r="B13">
         <v>15.846153846153847</v>
       </c>
     </row>
@@ -34859,7 +35200,7 @@
       <c r="A14" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B14" s="7">
+      <c r="B14">
         <v>15.571428571428571</v>
       </c>
     </row>
@@ -34867,7 +35208,7 @@
       <c r="A15" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B15" s="7">
+      <c r="B15">
         <v>17.642857142857142</v>
       </c>
     </row>
@@ -34875,7 +35216,7 @@
       <c r="A16" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B16" s="7">
+      <c r="B16">
         <v>20.23076923076923</v>
       </c>
     </row>
@@ -34883,7 +35224,7 @@
       <c r="A17" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B17" s="7">
+      <c r="B17">
         <v>15.642857142857142</v>
       </c>
     </row>
@@ -34891,7 +35232,7 @@
       <c r="A18" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B18" s="7">
+      <c r="B18">
         <v>16.866666666666667</v>
       </c>
     </row>
@@ -34899,7 +35240,7 @@
       <c r="A19" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B19" s="7">
+      <c r="B19">
         <v>19.23076923076923</v>
       </c>
     </row>
@@ -34907,7 +35248,7 @@
       <c r="A20" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B20" s="7">
+      <c r="B20">
         <v>21.23076923076923</v>
       </c>
     </row>
@@ -34915,7 +35256,7 @@
       <c r="A21" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B21" s="7">
+      <c r="B21">
         <v>37.75</v>
       </c>
     </row>
@@ -34923,7 +35264,7 @@
       <c r="A22" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B22" s="7">
+      <c r="B22">
         <v>32.222222222222221</v>
       </c>
     </row>
@@ -34931,7 +35272,7 @@
       <c r="A23" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B23" s="7">
+      <c r="B23">
         <v>25.833333333333332</v>
       </c>
     </row>
@@ -34939,7 +35280,7 @@
       <c r="A24" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B24" s="7">
+      <c r="B24">
         <v>42.375</v>
       </c>
     </row>
@@ -34947,7 +35288,7 @@
       <c r="A25" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B25" s="7">
+      <c r="B25">
         <v>24.166666666666668</v>
       </c>
     </row>
@@ -34955,7 +35296,7 @@
       <c r="A26" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B26" s="7">
+      <c r="B26">
         <v>20.636363636363637</v>
       </c>
     </row>
@@ -34963,7 +35304,7 @@
       <c r="A27" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B27" s="7">
+      <c r="B27">
         <v>28.857142857142858</v>
       </c>
     </row>
@@ -34971,7 +35312,7 @@
       <c r="A28" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B28" s="7">
+      <c r="B28">
         <v>31</v>
       </c>
     </row>
@@ -34979,7 +35320,7 @@
       <c r="A29" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B29" s="7">
+      <c r="B29">
         <v>30.333333333333332</v>
       </c>
     </row>
@@ -34987,7 +35328,7 @@
       <c r="A30" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B30" s="7">
+      <c r="B30">
         <v>41.5</v>
       </c>
     </row>
@@ -34995,7 +35336,7 @@
       <c r="A31" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="B31" s="7">
+      <c r="B31">
         <v>36</v>
       </c>
     </row>
@@ -35003,7 +35344,7 @@
       <c r="A32" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B32" s="7">
+      <c r="B32">
         <v>18.508710801393729</v>
       </c>
     </row>
@@ -35039,15 +35380,11 @@
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
@@ -35075,8 +35412,6 @@
       <c r="A6" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
@@ -35115,8 +35450,6 @@
       <c r="A10" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
@@ -35155,8 +35488,6 @@
       <c r="A14" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
@@ -35184,15 +35515,11 @@
       <c r="A17" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
@@ -35220,8 +35547,6 @@
       <c r="A21" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="B21" s="7"/>
-      <c r="C21" s="7"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
@@ -35249,8 +35574,6 @@
       <c r="A24" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="B24" s="7"/>
-      <c r="C24" s="7"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
@@ -35278,8 +35601,6 @@
       <c r="A27" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="B27" s="7"/>
-      <c r="C27" s="7"/>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
@@ -35338,7 +35659,7 @@
       <c r="B2" s="5">
         <v>0.44833759590792838</v>
       </c>
-      <c r="C2" s="7">
+      <c r="C2">
         <v>22.692165044042653</v>
       </c>
     </row>
@@ -35349,7 +35670,7 @@
       <c r="B3" s="5">
         <v>0.43169697798441131</v>
       </c>
-      <c r="C3" s="7">
+      <c r="C3">
         <v>21.970163618864294</v>
       </c>
     </row>
@@ -35360,7 +35681,7 @@
       <c r="B4" s="5">
         <v>0.43795322234705342</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4">
         <v>23.093403598037433</v>
       </c>
     </row>
@@ -35371,7 +35692,7 @@
       <c r="B5" s="5">
         <v>0.36974938228026827</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5">
         <v>20.745169420330441</v>
       </c>
     </row>
@@ -35382,7 +35703,7 @@
       <c r="B6" s="5">
         <v>0.28947368421052633</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6">
         <v>16.462962962962962</v>
       </c>
     </row>
@@ -35393,7 +35714,7 @@
       <c r="B7" s="5">
         <v>0.42289579907310509</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7">
         <v>22.168771452626125</v>
       </c>
     </row>
@@ -35415,7 +35736,7 @@
       <c r="B13" s="5">
         <v>7.1859063514140009E-2</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="7">
         <v>204.97563624511076</v>
       </c>
     </row>
@@ -35426,7 +35747,7 @@
       <c r="B14" s="5">
         <v>9.3840230991337828E-2</v>
       </c>
-      <c r="C14" s="8">
+      <c r="C14" s="7">
         <v>205.16611265899439</v>
       </c>
     </row>
@@ -35437,7 +35758,7 @@
       <c r="B15" s="5">
         <v>7.8502634926403775E-2</v>
       </c>
-      <c r="C15" s="8">
+      <c r="C15" s="7">
         <v>203.2058367206337</v>
       </c>
     </row>
@@ -35448,7 +35769,7 @@
       <c r="B16" s="5">
         <v>4.2005040604872583E-2</v>
       </c>
-      <c r="C16" s="8">
+      <c r="C16" s="7">
         <v>204.29969566736577</v>
       </c>
     </row>
@@ -35459,7 +35780,7 @@
       <c r="B17" s="5">
         <v>1.8518518518518517E-2</v>
       </c>
-      <c r="C17" s="8">
+      <c r="C17" s="7">
         <v>200.14666666666656</v>
       </c>
     </row>
@@ -35470,7 +35791,7 @@
       <c r="B18" s="5">
         <v>7.3052263454439478E-2</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C18" s="7">
         <v>204.11633034415902</v>
       </c>
     </row>
@@ -35551,13 +35872,13 @@
       <c r="A6" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6">
         <v>232</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6">
         <v>70</v>
       </c>
     </row>
@@ -35565,13 +35886,13 @@
       <c r="A7" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7">
         <v>70</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="G7" s="7">
+      <c r="G7">
         <v>47</v>
       </c>
     </row>
@@ -35579,13 +35900,13 @@
       <c r="A8" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8">
         <v>64</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="G8" s="7">
+      <c r="G8">
         <v>37</v>
       </c>
     </row>
@@ -35593,13 +35914,13 @@
       <c r="A9" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B9">
         <v>33</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="G9" s="7">
+      <c r="G9">
         <v>35</v>
       </c>
     </row>
@@ -35607,13 +35928,13 @@
       <c r="A10" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B10" s="7">
+      <c r="B10">
         <v>31</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="G10" s="7">
+      <c r="G10">
         <v>30</v>
       </c>
     </row>
@@ -35621,13 +35942,13 @@
       <c r="A11" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B11" s="7">
+      <c r="B11">
         <v>26</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="G11" s="7">
+      <c r="G11">
         <v>25</v>
       </c>
     </row>
@@ -35635,13 +35956,13 @@
       <c r="A12" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B12" s="7">
+      <c r="B12">
         <v>20</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="G12" s="7">
+      <c r="G12">
         <v>17</v>
       </c>
     </row>
@@ -35649,13 +35970,13 @@
       <c r="A13" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="B13" s="7">
+      <c r="B13">
         <v>17</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="G13" s="7">
+      <c r="G13">
         <v>15</v>
       </c>
     </row>
@@ -35663,13 +35984,13 @@
       <c r="A14" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B14" s="7">
+      <c r="B14">
         <v>16</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="G14" s="7">
+      <c r="G14">
         <v>12</v>
       </c>
     </row>
@@ -35677,13 +35998,13 @@
       <c r="A15" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="B15" s="7">
+      <c r="B15">
         <v>15</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="G15" s="7">
+      <c r="G15">
         <v>9</v>
       </c>
     </row>
@@ -35691,13 +36012,13 @@
       <c r="A16" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="7">
+      <c r="B16">
         <v>524</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="G16" s="7">
+      <c r="G16">
         <v>297</v>
       </c>
     </row>
@@ -35763,22 +36084,22 @@
       <c r="A4" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="B4" s="7">
+      <c r="B4">
         <v>5</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4">
         <v>121</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D4">
         <v>2</v>
       </c>
-      <c r="E4" s="7">
+      <c r="E4">
         <v>46</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4">
         <v>7</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4">
         <v>167</v>
       </c>
     </row>
@@ -35786,22 +36107,22 @@
       <c r="A5" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5">
         <v>3</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5">
         <v>132</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5">
         <v>6</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5">
         <v>39</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5">
         <v>9</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5">
         <v>171</v>
       </c>
     </row>
@@ -35809,18 +36130,16 @@
       <c r="A6" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6">
         <v>1</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6">
         <v>5</v>
       </c>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7">
+      <c r="F6">
         <v>1</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6">
         <v>5</v>
       </c>
     </row>
@@ -35828,22 +36147,22 @@
       <c r="A7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7">
         <v>9</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7">
         <v>258</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7">
         <v>8</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7">
         <v>85</v>
       </c>
-      <c r="F7" s="7">
+      <c r="F7">
         <v>17</v>
       </c>
-      <c r="G7" s="7">
+      <c r="G7">
         <v>343</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: done with report
</commit_message>
<xml_diff>
--- a/project/stage03/analysis.xlsx
+++ b/project/stage03/analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jantar\uni-data-warehouse\project\stage03\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5540BB3B-B167-420C-9801-3F7FFF8E1AFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D88B6B9-DBBF-4A54-888D-5003CFA5D985}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="879" firstSheet="4" activeTab="10" xr2:uid="{5D7D4CC1-6A94-48C8-A9CB-AB14AE6EE489}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="879" firstSheet="5" activeTab="8" xr2:uid="{5D7D4CC1-6A94-48C8-A9CB-AB14AE6EE489}"/>
   </bookViews>
   <sheets>
     <sheet name="RainVsPitStops" sheetId="1" r:id="rId1"/>
@@ -27,21 +27,21 @@
   </sheets>
   <calcPr calcId="0"/>
   <pivotCaches>
-    <pivotCache cacheId="132" r:id="rId12"/>
-    <pivotCache cacheId="135" r:id="rId13"/>
-    <pivotCache cacheId="138" r:id="rId14"/>
-    <pivotCache cacheId="141" r:id="rId15"/>
-    <pivotCache cacheId="144" r:id="rId16"/>
-    <pivotCache cacheId="147" r:id="rId17"/>
-    <pivotCache cacheId="150" r:id="rId18"/>
-    <pivotCache cacheId="153" r:id="rId19"/>
-    <pivotCache cacheId="156" r:id="rId20"/>
-    <pivotCache cacheId="159" r:id="rId21"/>
-    <pivotCache cacheId="162" r:id="rId22"/>
-    <pivotCache cacheId="165" r:id="rId23"/>
-    <pivotCache cacheId="168" r:id="rId24"/>
-    <pivotCache cacheId="171" r:id="rId25"/>
-    <pivotCache cacheId="174" r:id="rId26"/>
+    <pivotCache cacheId="0" r:id="rId12"/>
+    <pivotCache cacheId="1" r:id="rId13"/>
+    <pivotCache cacheId="2" r:id="rId14"/>
+    <pivotCache cacheId="3" r:id="rId15"/>
+    <pivotCache cacheId="4" r:id="rId16"/>
+    <pivotCache cacheId="5" r:id="rId17"/>
+    <pivotCache cacheId="6" r:id="rId18"/>
+    <pivotCache cacheId="7" r:id="rId19"/>
+    <pivotCache cacheId="8" r:id="rId20"/>
+    <pivotCache cacheId="9" r:id="rId21"/>
+    <pivotCache cacheId="10" r:id="rId22"/>
+    <pivotCache cacheId="11" r:id="rId23"/>
+    <pivotCache cacheId="12" r:id="rId24"/>
+    <pivotCache cacheId="13" r:id="rId25"/>
+    <pivotCache cacheId="17" r:id="rId26"/>
   </pivotCaches>
 </workbook>
 </file>
@@ -3619,10 +3619,10 @@
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
+                  <c:v>Calm</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>Light Breeze</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Calm</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>Moderate Breeze</c:v>
@@ -3637,10 +3637,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>5</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1</c:v>
@@ -3684,10 +3684,10 @@
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
+                  <c:v>Calm</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>Light Breeze</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Calm</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>Moderate Breeze</c:v>
@@ -3702,10 +3702,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
+                  <c:v>132</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>121</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>132</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>5</c:v>
@@ -3749,10 +3749,10 @@
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
+                  <c:v>Calm</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>Light Breeze</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Calm</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>Moderate Breeze</c:v>
@@ -3767,10 +3767,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>6</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3811,10 +3811,10 @@
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
+                  <c:v>Calm</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>Light Breeze</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Calm</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>Moderate Breeze</c:v>
@@ -3829,10 +3829,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
+                  <c:v>39</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>46</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>39</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -27267,7 +27267,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition15.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="Jantar" refreshedDate="45809.650491319444" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{7D06339B-CF30-4D37-AE3F-EEB11A431A55}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshedBy="Jantar" refreshedDate="45809.69535613426" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="0" supportSubquery="1" supportAdvancedDrill="1" xr:uid="{7D06339B-CF30-4D37-AE3F-EEB11A431A55}">
   <cacheSource type="external" connectionId="1"/>
   <cacheFields count="5">
     <cacheField name="[Dim Weather].[Did Rain Occur].[Did Rain Occur]" caption="Did Rain Occur" numFmtId="0" hierarchy="39" level="1">
@@ -28925,7 +28925,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{56F7BB47-9FE9-44F6-BAE3-68381FD572F9}" name="PivotTable1" cacheId="144" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{56F7BB47-9FE9-44F6-BAE3-68381FD572F9}" name="PivotTable1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" fieldListSortAscending="1">
   <location ref="A4:D12" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="7">
     <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
@@ -29187,7 +29187,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable10.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{64550925-18BC-4527-BBCE-E54A3262D0D6}" name="PivotTable1" cacheId="165" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{64550925-18BC-4527-BBCE-E54A3262D0D6}" name="PivotTable1" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" fieldListSortAscending="1">
   <location ref="A1:C7" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -29364,350 +29364,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable11.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5AA7137E-FDF2-411F-A7E9-D7AEEDDD54ED}" name="PivotTable4" cacheId="171" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1" fieldListSortAscending="1">
-  <location ref="F5:G16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="3" colPageCount="1"/>
-  <pivotFields count="5">
-    <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" measureFilter="1" sortType="descending" defaultSubtotal="0" defaultAttributeDrillState="1">
-      <items count="10">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-      </items>
-      <autoSortScope>
-        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
-          <references count="1">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </autoSortScope>
-    </pivotField>
-    <pivotField axis="axisPage" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1"/>
-    <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField axis="axisPage" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1"/>
-    <pivotField axis="axisPage" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="11">
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <pageFields count="3">
-    <pageField fld="1" hier="25" name="[Dim Status].[Status Category].&amp;[Mechanical Failure]" cap="Mechanical Failure"/>
-    <pageField fld="3" hier="37" name="[Dim Time].[Year].&amp;[2010]" cap="2010"/>
-    <pageField fld="4" hier="12" name="[Dim Constructor].[Continent].&amp;[Europe]" cap="Europe"/>
-  </pageFields>
-  <dataFields count="1">
-    <dataField fld="2" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="11">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="2">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="3">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="4">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="8"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="5">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="6"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="6">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="4"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="7">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="9"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="8">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="9">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="7"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="10">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="5"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotHierarchies count="83">
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy multipleItemSelectionAllowed="1">
-      <members count="1" level="1">
-        <member name="[Dim Constructor].[Continent].&amp;[Europe]"/>
-      </members>
-    </pivotHierarchy>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy multipleItemSelectionAllowed="1">
-      <members count="1" level="1">
-        <member name="[Dim Status].[Status Category].&amp;[Mechanical Failure]"/>
-      </members>
-    </pivotHierarchy>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy multipleItemSelectionAllowed="1">
-      <members count="11" level="1">
-        <member name="[Dim Time].[Year].&amp;[2010]"/>
-        <member name="[Dim Time].[Year].&amp;[2011]"/>
-        <member name="[Dim Time].[Year].&amp;[2012]"/>
-        <member name="[Dim Time].[Year].&amp;[2013]"/>
-        <member name="[Dim Time].[Year].&amp;[2014]"/>
-        <member name="[Dim Time].[Year].&amp;[2015]"/>
-        <member name="[Dim Time].[Year].&amp;[2016]"/>
-        <member name="[Dim Time].[Year].&amp;[2017]"/>
-        <member name="[Dim Time].[Year].&amp;[2018]"/>
-        <member name="[Dim Time].[Year].&amp;[2019]"/>
-        <member name="[Dim Time].[Year].&amp;[2020]"/>
-      </members>
-    </pivotHierarchy>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
-    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragOff="0"/>
-  </pivotHierarchies>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <filters count="1">
-    <filter fld="0" type="count" id="1" iMeasureHier="53">
-      <autoFilter ref="A1">
-        <filterColumn colId="0">
-          <top10 val="10" filterVal="10"/>
-        </filterColumn>
-      </autoFilter>
-    </filter>
-  </filters>
-  <rowHierarchiesUsage count="1">
-    <rowHierarchyUsage hierarchyUsage="26"/>
-  </rowHierarchiesUsage>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" calculatedMembersInFilters="1" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable12.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A746FFF8-6B66-4252-8CEA-043143963F3D}" name="PivotTable3" cacheId="168" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A746FFF8-6B66-4252-8CEA-043143963F3D}" name="PivotTable3" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1" fieldListSortAscending="1">
   <location ref="A5:B16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="3" colPageCount="1"/>
   <pivotFields count="6">
     <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" measureFilter="1" sortType="descending" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -30054,8 +29711,351 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable12.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5AA7137E-FDF2-411F-A7E9-D7AEEDDD54ED}" name="PivotTable4" cacheId="13" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1" fieldListSortAscending="1">
+  <location ref="F5:G16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="3" colPageCount="1"/>
+  <pivotFields count="5">
+    <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" measureFilter="1" sortType="descending" defaultSubtotal="0" defaultAttributeDrillState="1">
+      <items count="10">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField axis="axisPage" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1"/>
+    <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField axis="axisPage" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1"/>
+    <pivotField axis="axisPage" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="11">
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <pageFields count="3">
+    <pageField fld="1" hier="25" name="[Dim Status].[Status Category].&amp;[Mechanical Failure]" cap="Mechanical Failure"/>
+    <pageField fld="3" hier="37" name="[Dim Time].[Year].&amp;[2010]" cap="2010"/>
+    <pageField fld="4" hier="12" name="[Dim Constructor].[Continent].&amp;[Europe]" cap="Europe"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField fld="2" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="11">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="2">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="3">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="4">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="8"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="5">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="6"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="6">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="7">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="9"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="8">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="9">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="7"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="10">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="5"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotHierarchies count="83">
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy multipleItemSelectionAllowed="1">
+      <members count="1" level="1">
+        <member name="[Dim Constructor].[Continent].&amp;[Europe]"/>
+      </members>
+    </pivotHierarchy>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy multipleItemSelectionAllowed="1">
+      <members count="1" level="1">
+        <member name="[Dim Status].[Status Category].&amp;[Mechanical Failure]"/>
+      </members>
+    </pivotHierarchy>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy multipleItemSelectionAllowed="1">
+      <members count="11" level="1">
+        <member name="[Dim Time].[Year].&amp;[2010]"/>
+        <member name="[Dim Time].[Year].&amp;[2011]"/>
+        <member name="[Dim Time].[Year].&amp;[2012]"/>
+        <member name="[Dim Time].[Year].&amp;[2013]"/>
+        <member name="[Dim Time].[Year].&amp;[2014]"/>
+        <member name="[Dim Time].[Year].&amp;[2015]"/>
+        <member name="[Dim Time].[Year].&amp;[2016]"/>
+        <member name="[Dim Time].[Year].&amp;[2017]"/>
+        <member name="[Dim Time].[Year].&amp;[2018]"/>
+        <member name="[Dim Time].[Year].&amp;[2019]"/>
+        <member name="[Dim Time].[Year].&amp;[2020]"/>
+      </members>
+    </pivotHierarchy>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragToData="1"/>
+    <pivotHierarchy dragToRow="0" dragToCol="0" dragToPage="0" dragOff="0"/>
+  </pivotHierarchies>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <filters count="1">
+    <filter fld="0" type="count" id="1" iMeasureHier="53">
+      <autoFilter ref="A1">
+        <filterColumn colId="0">
+          <top10 val="10" filterVal="10"/>
+        </filterColumn>
+      </autoFilter>
+    </filter>
+  </filters>
+  <rowHierarchiesUsage count="1">
+    <rowHierarchyUsage hierarchyUsage="26"/>
+  </rowHierarchiesUsage>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" calculatedMembersInFilters="1" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/pivotTables/pivotTable13.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8EE1C926-7098-4912-8FCE-3C5B6C4A9ADA}" name="PivotTable5" cacheId="174" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8EE1C926-7098-4912-8FCE-3C5B6C4A9ADA}" name="PivotTable5" cacheId="17" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3" fieldListSortAscending="1">
   <location ref="A1:G7" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisCol" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -30076,8 +30076,8 @@
     </pivotField>
     <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" defaultSubtotal="0" defaultAttributeDrillState="1">
       <items count="3">
+        <item x="0"/>
         <item x="1"/>
-        <item x="0"/>
         <item x="2"/>
       </items>
     </pivotField>
@@ -30310,7 +30310,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable14.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8B5532C8-184E-45A3-9671-D5D71185BFA5}" name="PivotTable6" cacheId="135" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8B5532C8-184E-45A3-9671-D5D71185BFA5}" name="PivotTable6" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1" fieldListSortAscending="1">
   <location ref="A3:B78" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="3">
     <pivotField axis="axisPage" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1"/>
@@ -30749,7 +30749,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable15.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FB381D15-99CD-4BB2-BFAA-5B743EDB0261}" name="PivotTable1" cacheId="132" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FB381D15-99CD-4BB2-BFAA-5B743EDB0261}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" fieldListSortAscending="1">
   <location ref="A3:E29" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
@@ -30893,23 +30893,23 @@
     <dataField name="Constructor Reliability KPI Trend" fld="3" baseField="0" baseItem="0"/>
   </dataFields>
   <conditionalFormats count="2">
+    <conditionalFormat scope="data" priority="1">
+      <pivotAreas count="1">
+        <pivotArea outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="3"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </pivotAreas>
+    </conditionalFormat>
     <conditionalFormat scope="data" priority="2">
       <pivotAreas count="1">
         <pivotArea outline="0" fieldPosition="0">
           <references count="1">
             <reference field="4294967294" count="1" selected="0">
               <x v="2"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </pivotAreas>
-    </conditionalFormat>
-    <conditionalFormat scope="data" priority="1">
-      <pivotAreas count="1">
-        <pivotArea outline="0" fieldPosition="0">
-          <references count="1">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="3"/>
             </reference>
           </references>
         </pivotArea>
@@ -31020,7 +31020,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C46A81BC-8C75-4F76-8210-EEF5A83AF696}" name="PivotTable4" cacheId="141" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C46A81BC-8C75-4F76-8210-EEF5A83AF696}" name="PivotTable4" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10" fieldListSortAscending="1">
   <location ref="A4:B22" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="7">
     <pivotField axis="axisPage" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1"/>
@@ -31579,7 +31579,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{48529DB8-E948-488C-A714-CF42C15C483B}" name="PivotTable2" cacheId="153" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{48529DB8-E948-488C-A714-CF42C15C483B}" name="PivotTable2" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" fieldListSortAscending="1">
   <location ref="F34:G58" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="3">
     <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
@@ -31837,7 +31837,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0D28268D-F139-414C-88E2-408A6595ABF9}" name="PivotTable5" cacheId="156" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="15" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0D28268D-F139-414C-88E2-408A6595ABF9}" name="PivotTable5" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="15" fieldListSortAscending="1">
   <location ref="A3:G5" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="3">
     <pivotField dataField="1" subtotalTop="0" showAll="0" defaultSubtotal="0"/>
@@ -32096,7 +32096,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F77C5366-9A19-47B5-8C19-F54DD5D444B7}" name="PivotTable4" cacheId="147" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F77C5366-9A19-47B5-8C19-F54DD5D444B7}" name="PivotTable4" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11" fieldListSortAscending="1">
   <location ref="K5:U14" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
   <pivotFields count="5">
     <pivotField axis="axisPage" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -32453,7 +32453,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2F74144B-8497-4A58-998A-35E2F835E367}" name="PivotTable1" cacheId="150" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2F74144B-8497-4A58-998A-35E2F835E367}" name="PivotTable1" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" subtotalHiddenItems="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" fieldListSortAscending="1">
   <location ref="A4:B31" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
   <pivotFields count="4">
     <pivotField axis="axisPage" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -32719,7 +32719,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FA00D414-BC42-451C-9F10-3DB99A7CAD38}" name="PivotTable3" cacheId="159" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FA00D414-BC42-451C-9F10-3DB99A7CAD38}" name="PivotTable3" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1" fieldListSortAscending="1">
   <location ref="A5:B32" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
   <pivotFields count="4">
     <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -33032,7 +33032,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F4BABA1E-A83D-4CB8-B63A-6BD641FCE2BF}" name="PivotTable1" cacheId="162" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F4BABA1E-A83D-4CB8-B63A-6BD641FCE2BF}" name="PivotTable1" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" fieldListSortAscending="1">
   <location ref="A1:C29" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" dataSourceSort="1" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -33291,7 +33291,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7F60A7DA-9FE7-47E8-A86B-C8A0C2243D7A}" name="PivotTable2" cacheId="138" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" fieldListSortAscending="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7F60A7DA-9FE7-47E8-A86B-C8A0C2243D7A}" name="PivotTable2" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="2" fieldListSortAscending="1">
   <location ref="A12:C18" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField axis="axisRow" allDrilled="1" subtotalTop="0" showAll="0" defaultSubtotal="0" defaultAttributeDrillState="1">
@@ -33845,13 +33845,13 @@
       <c r="A6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6">
         <v>1.4611872146118721</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6">
         <v>1.3251533742331287</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6">
         <v>1.4031413612565444</v>
       </c>
     </row>
@@ -33859,13 +33859,13 @@
       <c r="A7" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7">
         <v>1.4928774928774928</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7">
         <v>2.1724137931034484</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7">
         <v>1.5892420537897312</v>
       </c>
     </row>
@@ -33873,13 +33873,13 @@
       <c r="A8" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="8">
+      <c r="B8">
         <v>1.904040404040404</v>
       </c>
-      <c r="C8" s="8">
+      <c r="C8">
         <v>1.9661016949152543</v>
       </c>
-      <c r="D8" s="8">
+      <c r="D8">
         <v>1.9182879377431907</v>
       </c>
     </row>
@@ -33887,13 +33887,13 @@
       <c r="A9" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B9">
         <v>1.9824561403508771</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9">
         <v>2.36</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9">
         <v>2.0611111111111109</v>
       </c>
     </row>
@@ -33901,13 +33901,13 @@
       <c r="A10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10">
         <v>1.9039735099337749</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10">
         <v>2.1296296296296298</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10">
         <v>1.9634146341463414</v>
       </c>
     </row>
@@ -33915,13 +33915,13 @@
       <c r="A11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="8">
+      <c r="B11">
         <v>1.8850931677018634</v>
       </c>
-      <c r="C11" s="8">
+      <c r="C11">
         <v>3.2105263157894739</v>
       </c>
-      <c r="D11" s="8">
+      <c r="D11">
         <v>2.1870503597122304</v>
       </c>
     </row>
@@ -33929,13 +33929,13 @@
       <c r="A12" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="8">
+      <c r="B12">
         <v>1.7698270721526534</v>
       </c>
-      <c r="C12" s="8">
+      <c r="C12">
         <v>2.096774193548387</v>
       </c>
-      <c r="D12" s="8">
+      <c r="D12">
         <v>1.8514541387024608</v>
       </c>
     </row>
@@ -34613,13 +34613,13 @@
       <c r="B4" s="5">
         <v>0.58981233243967823</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4">
         <v>0.8</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4">
         <v>-1</v>
       </c>
-      <c r="E4" s="8">
+      <c r="E4">
         <v>1</v>
       </c>
     </row>
@@ -34630,13 +34630,13 @@
       <c r="B5" s="5">
         <v>0.5802139037433155</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5">
         <v>0.8</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5">
         <v>-1</v>
       </c>
-      <c r="E5" s="8">
+      <c r="E5">
         <v>-1</v>
       </c>
     </row>
@@ -34647,13 +34647,13 @@
       <c r="B6" s="5">
         <v>0.55524861878453047</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6">
         <v>0.8</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6">
         <v>-1</v>
       </c>
-      <c r="E6" s="8">
+      <c r="E6">
         <v>-1</v>
       </c>
     </row>
@@ -34664,13 +34664,13 @@
       <c r="B7" s="5">
         <v>0.65312499999999996</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7">
         <v>0.8</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7">
         <v>-1</v>
       </c>
-      <c r="E7" s="8">
+      <c r="E7">
         <v>1</v>
       </c>
     </row>
@@ -34681,13 +34681,13 @@
       <c r="B8" s="5">
         <v>0.71944444444444444</v>
       </c>
-      <c r="C8" s="8">
+      <c r="C8">
         <v>0.8</v>
       </c>
-      <c r="D8" s="8">
+      <c r="D8">
         <v>-1</v>
       </c>
-      <c r="E8" s="8">
+      <c r="E8">
         <v>1</v>
       </c>
     </row>
@@ -34698,13 +34698,13 @@
       <c r="B9" s="5">
         <v>0.7393617021276595</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9">
         <v>0.8</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9">
         <v>0</v>
       </c>
-      <c r="E9" s="8">
+      <c r="E9">
         <v>1</v>
       </c>
     </row>
@@ -34715,13 +34715,13 @@
       <c r="B10" s="5">
         <v>0.67929292929292928</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10">
         <v>0.8</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10">
         <v>-1</v>
       </c>
-      <c r="E10" s="8">
+      <c r="E10">
         <v>-1</v>
       </c>
     </row>
@@ -34732,13 +34732,13 @@
       <c r="B11" s="5">
         <v>0.73262032085561501</v>
       </c>
-      <c r="C11" s="8">
+      <c r="C11">
         <v>0.8</v>
       </c>
-      <c r="D11" s="8">
+      <c r="D11">
         <v>0</v>
       </c>
-      <c r="E11" s="8">
+      <c r="E11">
         <v>1</v>
       </c>
     </row>
@@ -34749,13 +34749,13 @@
       <c r="B12" s="5">
         <v>0.76358695652173914</v>
       </c>
-      <c r="C12" s="8">
+      <c r="C12">
         <v>0.8</v>
       </c>
-      <c r="D12" s="8">
+      <c r="D12">
         <v>0</v>
       </c>
-      <c r="E12" s="8">
+      <c r="E12">
         <v>1</v>
       </c>
     </row>
@@ -34766,13 +34766,13 @@
       <c r="B13" s="5">
         <v>0.80294117647058827</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13">
         <v>0.8</v>
       </c>
-      <c r="D13" s="8">
+      <c r="D13">
         <v>1</v>
       </c>
-      <c r="E13" s="8">
+      <c r="E13">
         <v>1</v>
       </c>
     </row>
@@ -34783,13 +34783,13 @@
       <c r="B14" s="5">
         <v>0.74780701754385959</v>
       </c>
-      <c r="C14" s="8">
+      <c r="C14">
         <v>0.8</v>
       </c>
-      <c r="D14" s="8">
+      <c r="D14">
         <v>0</v>
       </c>
-      <c r="E14" s="8">
+      <c r="E14">
         <v>-1</v>
       </c>
     </row>
@@ -34800,13 +34800,13 @@
       <c r="B15" s="5">
         <v>0.83114035087719296</v>
       </c>
-      <c r="C15" s="8">
+      <c r="C15">
         <v>0.8</v>
       </c>
-      <c r="D15" s="8">
+      <c r="D15">
         <v>1</v>
       </c>
-      <c r="E15" s="8">
+      <c r="E15">
         <v>1</v>
       </c>
     </row>
@@ -34817,13 +34817,13 @@
       <c r="B16" s="5">
         <v>0.82291666666666663</v>
       </c>
-      <c r="C16" s="8">
+      <c r="C16">
         <v>0.8</v>
       </c>
-      <c r="D16" s="8">
+      <c r="D16">
         <v>1</v>
       </c>
-      <c r="E16" s="8">
+      <c r="E16">
         <v>-1</v>
       </c>
     </row>
@@ -34834,13 +34834,13 @@
       <c r="B17" s="5">
         <v>0.85406698564593297</v>
       </c>
-      <c r="C17" s="8">
+      <c r="C17">
         <v>0.8</v>
       </c>
-      <c r="D17" s="8">
+      <c r="D17">
         <v>1</v>
       </c>
-      <c r="E17" s="8">
+      <c r="E17">
         <v>1</v>
       </c>
     </row>
@@ -34851,13 +34851,13 @@
       <c r="B18" s="5">
         <v>0.80835380835380832</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C18">
         <v>0.8</v>
       </c>
-      <c r="D18" s="8">
+      <c r="D18">
         <v>1</v>
       </c>
-      <c r="E18" s="8">
+      <c r="E18">
         <v>-1</v>
       </c>
     </row>
@@ -34868,13 +34868,13 @@
       <c r="B19" s="5">
         <v>0.81746031746031744</v>
       </c>
-      <c r="C19" s="8">
+      <c r="C19">
         <v>0.8</v>
       </c>
-      <c r="D19" s="8">
+      <c r="D19">
         <v>1</v>
       </c>
-      <c r="E19" s="8">
+      <c r="E19">
         <v>1</v>
       </c>
     </row>
@@ -34885,13 +34885,13 @@
       <c r="B20" s="5">
         <v>0.83982683982683981</v>
       </c>
-      <c r="C20" s="8">
+      <c r="C20">
         <v>0.8</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D20">
         <v>1</v>
       </c>
-      <c r="E20" s="8">
+      <c r="E20">
         <v>1</v>
       </c>
     </row>
@@ -34902,13 +34902,13 @@
       <c r="B21" s="5">
         <v>0.76249999999999996</v>
       </c>
-      <c r="C21" s="8">
+      <c r="C21">
         <v>0.8</v>
       </c>
-      <c r="D21" s="8">
+      <c r="D21">
         <v>0</v>
       </c>
-      <c r="E21" s="8">
+      <c r="E21">
         <v>-1</v>
       </c>
     </row>
@@ -34919,13 +34919,13 @@
       <c r="B22" s="5">
         <v>0.80238095238095242</v>
       </c>
-      <c r="C22" s="8">
+      <c r="C22">
         <v>0.8</v>
       </c>
-      <c r="D22" s="8">
+      <c r="D22">
         <v>1</v>
       </c>
-      <c r="E22" s="8">
+      <c r="E22">
         <v>1</v>
       </c>
     </row>
@@ -34936,13 +34936,13 @@
       <c r="B23" s="5">
         <v>0.86190476190476195</v>
       </c>
-      <c r="C23" s="8">
+      <c r="C23">
         <v>0.8</v>
       </c>
-      <c r="D23" s="8">
+      <c r="D23">
         <v>1</v>
       </c>
-      <c r="E23" s="8">
+      <c r="E23">
         <v>1</v>
       </c>
     </row>
@@ -34953,13 +34953,13 @@
       <c r="B24" s="5">
         <v>0.83529411764705885</v>
       </c>
-      <c r="C24" s="8">
+      <c r="C24">
         <v>0.8</v>
       </c>
-      <c r="D24" s="8">
+      <c r="D24">
         <v>1</v>
       </c>
-      <c r="E24" s="8">
+      <c r="E24">
         <v>-1</v>
       </c>
     </row>
@@ -34970,13 +34970,13 @@
       <c r="B25" s="5">
         <v>0.8727272727272728</v>
       </c>
-      <c r="C25" s="8">
+      <c r="C25">
         <v>0.8</v>
       </c>
-      <c r="D25" s="8">
+      <c r="D25">
         <v>1</v>
       </c>
-      <c r="E25" s="8">
+      <c r="E25">
         <v>1</v>
       </c>
     </row>
@@ -34987,13 +34987,13 @@
       <c r="B26" s="5">
         <v>0.83181818181818179</v>
       </c>
-      <c r="C26" s="8">
+      <c r="C26">
         <v>0.8</v>
       </c>
-      <c r="D26" s="8">
+      <c r="D26">
         <v>1</v>
       </c>
-      <c r="E26" s="8">
+      <c r="E26">
         <v>-1</v>
       </c>
     </row>
@@ -35004,13 +35004,13 @@
       <c r="B27" s="5">
         <v>0.85681818181818181</v>
       </c>
-      <c r="C27" s="8">
+      <c r="C27">
         <v>0.8</v>
       </c>
-      <c r="D27" s="8">
+      <c r="D27">
         <v>1</v>
       </c>
-      <c r="E27" s="8">
+      <c r="E27">
         <v>1</v>
       </c>
     </row>
@@ -35021,13 +35021,13 @@
       <c r="B28" s="5">
         <v>0.90605427974947805</v>
       </c>
-      <c r="C28" s="8">
+      <c r="C28">
         <v>0.8</v>
       </c>
-      <c r="D28" s="8">
+      <c r="D28">
         <v>1</v>
       </c>
-      <c r="E28" s="8">
+      <c r="E28">
         <v>1</v>
       </c>
     </row>
@@ -35038,13 +35038,13 @@
       <c r="B29" s="5">
         <v>0.77666435162218472</v>
       </c>
-      <c r="C29" s="8">
+      <c r="C29">
         <v>0.8</v>
       </c>
-      <c r="D29" s="8">
+      <c r="D29">
         <v>0</v>
       </c>
-      <c r="E29" s="8">
+      <c r="E29">
         <v>0</v>
       </c>
     </row>
@@ -35129,19 +35129,17 @@
       <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="8"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="8"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7">
         <v>1.2086570477247502</v>
       </c>
     </row>
@@ -35149,13 +35147,12 @@
       <c r="A8" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="8"/>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B9">
         <v>0.56140350877192979</v>
       </c>
     </row>
@@ -35163,7 +35160,7 @@
       <c r="A10" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10">
         <v>3.4645390070921986</v>
       </c>
     </row>
@@ -35171,7 +35168,7 @@
       <c r="A11" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="B11" s="8">
+      <c r="B11">
         <v>1.4308426073131955</v>
       </c>
     </row>
@@ -35179,13 +35176,12 @@
       <c r="A12" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="8"/>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13">
         <v>1.1666666666666667</v>
       </c>
     </row>
@@ -35193,7 +35189,7 @@
       <c r="A14" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="B14" s="8">
+      <c r="B14">
         <v>4.2163742690058479</v>
       </c>
     </row>
@@ -35201,7 +35197,7 @@
       <c r="A15" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="B15" s="8">
+      <c r="B15">
         <v>2.6777546777546779</v>
       </c>
     </row>
@@ -35209,7 +35205,7 @@
       <c r="A16" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="B16" s="8">
+      <c r="B16">
         <v>1.1880952380952381</v>
       </c>
     </row>
@@ -35217,7 +35213,7 @@
       <c r="A17" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="B17" s="8">
+      <c r="B17">
         <v>1.0948616600790513</v>
       </c>
     </row>
@@ -35225,7 +35221,7 @@
       <c r="A18" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="B18" s="8">
+      <c r="B18">
         <v>0.94680851063829785</v>
       </c>
     </row>
@@ -35233,13 +35229,12 @@
       <c r="A19" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="8"/>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="B20" s="8">
+      <c r="B20">
         <v>2.3026737967914439</v>
       </c>
     </row>
@@ -35247,7 +35242,7 @@
       <c r="A21" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="B21" s="8">
+      <c r="B21">
         <v>0.98565573770491799</v>
       </c>
     </row>
@@ -35255,7 +35250,7 @@
       <c r="A22" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B22" s="8">
+      <c r="B22">
         <v>1.6894683372841179</v>
       </c>
     </row>
@@ -35322,22 +35317,22 @@
       <c r="A5" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5">
         <v>4.5844155844155843</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5">
         <v>5.6934426229508199</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5">
         <v>9.9909836065573767</v>
       </c>
-      <c r="E5" s="8">
+      <c r="E5">
         <v>12.158196721311475</v>
       </c>
-      <c r="F5" s="8">
+      <c r="F5">
         <v>12.445081967213115</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5">
         <v>9.7461449498843482</v>
       </c>
     </row>
@@ -35381,7 +35376,7 @@
       <c r="F35" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G35" s="8">
+      <c r="G35">
         <v>12.445081967213115</v>
       </c>
       <c r="J35" s="2" t="s">
@@ -35395,7 +35390,7 @@
       <c r="F36" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="G36" s="8">
+      <c r="G36">
         <v>12.158196721311475</v>
       </c>
       <c r="J36" s="2" t="s">
@@ -35409,7 +35404,7 @@
       <c r="F37" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="G37" s="8">
+      <c r="G37">
         <v>9.9909836065573767</v>
       </c>
       <c r="J37" s="2" t="s">
@@ -35423,7 +35418,7 @@
       <c r="F38" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="G38" s="8">
+      <c r="G38">
         <v>5.6934426229508199</v>
       </c>
     </row>
@@ -35431,7 +35426,7 @@
       <c r="F39" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="G39" s="8">
+      <c r="G39">
         <v>4.5844155844155843</v>
       </c>
     </row>
@@ -35439,7 +35434,7 @@
       <c r="F40" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="G40" s="8">
+      <c r="G40">
         <v>3.7236842105263159</v>
       </c>
     </row>
@@ -35447,7 +35442,7 @@
       <c r="F41" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="G41" s="8">
+      <c r="G41">
         <v>3.0649717514124295</v>
       </c>
     </row>
@@ -35455,7 +35450,7 @@
       <c r="F42" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="G42" s="8">
+      <c r="G42">
         <v>2.7666666666666666</v>
       </c>
     </row>
@@ -35463,7 +35458,7 @@
       <c r="F43" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G43" s="8">
+      <c r="G43">
         <v>2.7333333333333334</v>
       </c>
     </row>
@@ -35471,7 +35466,7 @@
       <c r="F44" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="G44" s="8">
+      <c r="G44">
         <v>2.5181159420289854</v>
       </c>
     </row>
@@ -35479,7 +35474,7 @@
       <c r="F45" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="G45" s="8">
+      <c r="G45">
         <v>1.8433734939759037</v>
       </c>
     </row>
@@ -35487,7 +35482,7 @@
       <c r="F46" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="G46" s="8">
+      <c r="G46">
         <v>1.6995073891625616</v>
       </c>
     </row>
@@ -35495,7 +35490,7 @@
       <c r="F47" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="G47" s="8">
+      <c r="G47">
         <v>1.1212121212121211</v>
       </c>
     </row>
@@ -35503,7 +35498,7 @@
       <c r="F48" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="G48" s="8">
+      <c r="G48">
         <v>0.91044776119402981</v>
       </c>
     </row>
@@ -35511,7 +35506,7 @@
       <c r="F49" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="G49" s="8">
+      <c r="G49">
         <v>0.83333333333333337</v>
       </c>
     </row>
@@ -35519,7 +35514,7 @@
       <c r="F50" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="G50" s="8">
+      <c r="G50">
         <v>0.77105263157894732</v>
       </c>
     </row>
@@ -35527,7 +35522,7 @@
       <c r="F51" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G51" s="8">
+      <c r="G51">
         <v>0.70673076923076927</v>
       </c>
     </row>
@@ -35535,7 +35530,7 @@
       <c r="F52" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="G52" s="8">
+      <c r="G52">
         <v>1.834862385321101E-2</v>
       </c>
     </row>
@@ -35543,7 +35538,7 @@
       <c r="F53" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="G53" s="8">
+      <c r="G53">
         <v>1.282051282051282E-2</v>
       </c>
     </row>
@@ -35551,7 +35546,7 @@
       <c r="F54" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="G54" s="8">
+      <c r="G54">
         <v>0</v>
       </c>
     </row>
@@ -35559,7 +35554,7 @@
       <c r="F55" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="G55" s="8">
+      <c r="G55">
         <v>0</v>
       </c>
     </row>
@@ -35567,7 +35562,7 @@
       <c r="F56" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G56" s="8">
+      <c r="G56">
         <v>0</v>
       </c>
     </row>
@@ -35575,7 +35570,7 @@
       <c r="F57" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G57" s="8">
+      <c r="G57">
         <v>0</v>
       </c>
     </row>
@@ -35583,7 +35578,7 @@
       <c r="F58" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="G58" s="8">
+      <c r="G58">
         <v>4.8117619639527653</v>
       </c>
     </row>
@@ -36265,7 +36260,7 @@
       <c r="A6" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6">
         <v>7.333333333333333</v>
       </c>
     </row>
@@ -36273,7 +36268,7 @@
       <c r="A7" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7">
         <v>10.857142857142858</v>
       </c>
     </row>
@@ -36281,7 +36276,7 @@
       <c r="A8" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B8" s="8">
+      <c r="B8">
         <v>12.461538461538462</v>
       </c>
     </row>
@@ -36289,7 +36284,7 @@
       <c r="A9" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B9">
         <v>9.2666666666666675</v>
       </c>
     </row>
@@ -36297,7 +36292,7 @@
       <c r="A10" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10">
         <v>6.7058823529411766</v>
       </c>
     </row>
@@ -36305,7 +36300,7 @@
       <c r="A11" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B11" s="8">
+      <c r="B11">
         <v>10</v>
       </c>
     </row>
@@ -36313,7 +36308,7 @@
       <c r="A12" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B12" s="8">
+      <c r="B12">
         <v>22.181818181818183</v>
       </c>
     </row>
@@ -36321,7 +36316,7 @@
       <c r="A13" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13">
         <v>15.846153846153847</v>
       </c>
     </row>
@@ -36329,7 +36324,7 @@
       <c r="A14" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B14" s="8">
+      <c r="B14">
         <v>15.571428571428571</v>
       </c>
     </row>
@@ -36337,7 +36332,7 @@
       <c r="A15" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B15" s="8">
+      <c r="B15">
         <v>17.642857142857142</v>
       </c>
     </row>
@@ -36345,7 +36340,7 @@
       <c r="A16" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B16" s="8">
+      <c r="B16">
         <v>20.23076923076923</v>
       </c>
     </row>
@@ -36353,7 +36348,7 @@
       <c r="A17" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B17" s="8">
+      <c r="B17">
         <v>15.642857142857142</v>
       </c>
     </row>
@@ -36361,7 +36356,7 @@
       <c r="A18" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B18" s="8">
+      <c r="B18">
         <v>16.866666666666667</v>
       </c>
     </row>
@@ -36369,7 +36364,7 @@
       <c r="A19" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B19" s="8">
+      <c r="B19">
         <v>19.23076923076923</v>
       </c>
     </row>
@@ -36377,7 +36372,7 @@
       <c r="A20" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B20" s="8">
+      <c r="B20">
         <v>21.23076923076923</v>
       </c>
     </row>
@@ -36385,7 +36380,7 @@
       <c r="A21" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B21" s="8">
+      <c r="B21">
         <v>37.75</v>
       </c>
     </row>
@@ -36393,7 +36388,7 @@
       <c r="A22" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B22" s="8">
+      <c r="B22">
         <v>32.222222222222221</v>
       </c>
     </row>
@@ -36401,7 +36396,7 @@
       <c r="A23" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B23" s="8">
+      <c r="B23">
         <v>25.833333333333332</v>
       </c>
     </row>
@@ -36409,7 +36404,7 @@
       <c r="A24" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B24" s="8">
+      <c r="B24">
         <v>42.375</v>
       </c>
     </row>
@@ -36417,7 +36412,7 @@
       <c r="A25" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B25" s="8">
+      <c r="B25">
         <v>24.166666666666668</v>
       </c>
     </row>
@@ -36425,7 +36420,7 @@
       <c r="A26" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B26" s="8">
+      <c r="B26">
         <v>20.636363636363637</v>
       </c>
     </row>
@@ -36433,7 +36428,7 @@
       <c r="A27" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B27" s="8">
+      <c r="B27">
         <v>28.857142857142858</v>
       </c>
     </row>
@@ -36441,7 +36436,7 @@
       <c r="A28" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B28" s="8">
+      <c r="B28">
         <v>31</v>
       </c>
     </row>
@@ -36449,7 +36444,7 @@
       <c r="A29" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B29" s="8">
+      <c r="B29">
         <v>30.333333333333332</v>
       </c>
     </row>
@@ -36457,7 +36452,7 @@
       <c r="A30" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B30" s="8">
+      <c r="B30">
         <v>41.5</v>
       </c>
     </row>
@@ -36465,7 +36460,7 @@
       <c r="A31" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="B31" s="8">
+      <c r="B31">
         <v>36</v>
       </c>
     </row>
@@ -36473,7 +36468,7 @@
       <c r="A32" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B32" s="8">
+      <c r="B32">
         <v>18.508710801393729</v>
       </c>
     </row>
@@ -36509,15 +36504,11 @@
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
@@ -36545,8 +36536,6 @@
       <c r="A6" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
@@ -36585,8 +36574,6 @@
       <c r="A10" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
@@ -36625,8 +36612,6 @@
       <c r="A14" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
@@ -36654,15 +36639,11 @@
       <c r="A17" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
@@ -36690,8 +36671,6 @@
       <c r="A21" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="B21" s="8"/>
-      <c r="C21" s="8"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
@@ -36719,8 +36698,6 @@
       <c r="A24" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="B24" s="8"/>
-      <c r="C24" s="8"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
@@ -36748,8 +36725,6 @@
       <c r="A27" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="B27" s="8"/>
-      <c r="C27" s="8"/>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
@@ -36808,7 +36783,7 @@
       <c r="B2" s="5">
         <v>0.44833759590792838</v>
       </c>
-      <c r="C2" s="8">
+      <c r="C2">
         <v>22.692165044042653</v>
       </c>
     </row>
@@ -36819,7 +36794,7 @@
       <c r="B3" s="5">
         <v>0.43169697798441131</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3">
         <v>21.970163618864294</v>
       </c>
     </row>
@@ -36830,7 +36805,7 @@
       <c r="B4" s="5">
         <v>0.43795322234705342</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4">
         <v>23.093403598037433</v>
       </c>
     </row>
@@ -36841,7 +36816,7 @@
       <c r="B5" s="5">
         <v>0.36974938228026827</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5">
         <v>20.745169420330441</v>
       </c>
     </row>
@@ -36852,7 +36827,7 @@
       <c r="B6" s="5">
         <v>0.28947368421052633</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6">
         <v>16.462962962962962</v>
       </c>
     </row>
@@ -36863,7 +36838,7 @@
       <c r="B7" s="5">
         <v>0.42289579907310509</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7">
         <v>22.168771452626125</v>
       </c>
     </row>
@@ -37021,13 +36996,13 @@
       <c r="A6" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6">
         <v>232</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6">
         <v>70</v>
       </c>
     </row>
@@ -37035,13 +37010,13 @@
       <c r="A7" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7">
         <v>70</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="G7" s="8">
+      <c r="G7">
         <v>47</v>
       </c>
     </row>
@@ -37049,13 +37024,13 @@
       <c r="A8" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="B8" s="8">
+      <c r="B8">
         <v>64</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="G8" s="8">
+      <c r="G8">
         <v>37</v>
       </c>
     </row>
@@ -37063,13 +37038,13 @@
       <c r="A9" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B9">
         <v>33</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9">
         <v>35</v>
       </c>
     </row>
@@ -37077,13 +37052,13 @@
       <c r="A10" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10">
         <v>31</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="G10" s="8">
+      <c r="G10">
         <v>30</v>
       </c>
     </row>
@@ -37091,13 +37066,13 @@
       <c r="A11" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B11" s="8">
+      <c r="B11">
         <v>26</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="G11" s="8">
+      <c r="G11">
         <v>25</v>
       </c>
     </row>
@@ -37105,13 +37080,13 @@
       <c r="A12" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B12" s="8">
+      <c r="B12">
         <v>20</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="G12" s="8">
+      <c r="G12">
         <v>17</v>
       </c>
     </row>
@@ -37119,13 +37094,13 @@
       <c r="A13" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="B13" s="8">
+      <c r="B13">
         <v>17</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="G13" s="8">
+      <c r="G13">
         <v>15</v>
       </c>
     </row>
@@ -37133,13 +37108,13 @@
       <c r="A14" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B14" s="8">
+      <c r="B14">
         <v>16</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="G14" s="8">
+      <c r="G14">
         <v>12</v>
       </c>
     </row>
@@ -37147,13 +37122,13 @@
       <c r="A15" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="B15" s="8">
+      <c r="B15">
         <v>15</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="G15" s="8">
+      <c r="G15">
         <v>9</v>
       </c>
     </row>
@@ -37161,13 +37136,13 @@
       <c r="A16" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="8">
+      <c r="B16">
         <v>524</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="G16" s="8">
+      <c r="G16">
         <v>297</v>
       </c>
     </row>
@@ -37231,48 +37206,48 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B4" s="8">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C4" s="8">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="D4" s="8">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E4" s="8">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="F4" s="8">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G4" s="8">
-        <v>167</v>
+        <v>171</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B5" s="8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C5" s="8">
-        <v>132</v>
+        <v>121</v>
       </c>
       <c r="D5" s="8">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E5" s="8">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="F5" s="8">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G5" s="8">
-        <v>171</v>
+        <v>167</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>